<commit_message>
update v3 del JPser
</commit_message>
<xml_diff>
--- a/files/timeList.xlsx
+++ b/files/timeList.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mutsu\Pictures\BnSNEOtimeList\files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C60AD753-1507-4830-97D2-99680C6D8BE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{594A1B5D-C124-498B-AA1E-D8C3852E5366}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-60" yWindow="165" windowWidth="16425" windowHeight="15510" tabRatio="758" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="758" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="timeList" sheetId="15" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4064" uniqueCount="741">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3678" uniqueCount="741">
   <si>
     <t>日</t>
     <phoneticPr fontId="1"/>
@@ -6973,7 +6973,7 @@
         <v>474</v>
       </c>
       <c r="F106" s="136" t="s">
-        <v>173</v>
+        <v>304</v>
       </c>
       <c r="G106" s="137" t="s">
         <v>660</v>
@@ -11471,12 +11471,12 @@
   </sheetData>
   <autoFilter ref="B1:H169" xr:uid="{43214550-866B-4296-AF4D-B97EB9C891BA}"/>
   <phoneticPr fontId="1"/>
-  <conditionalFormatting sqref="C1:C1048576 L80:L81 N80:N81 P80:P81 E1:E1048576 G1:G1048576">
+  <conditionalFormatting sqref="C1:C1048576 E1:E1048576 G1:G1048576 L80:L81 N80:N81 P80:P81">
     <cfRule type="containsText" dxfId="7" priority="4" operator="containsText" text="'">
       <formula>NOT(ISERROR(SEARCH("'",C1)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D1:D1048576 M80:M81 O80:O81 Q80:Q81 F1:F1048576 H1:H1048576">
+  <conditionalFormatting sqref="D1:D1048576 F1:F1048576 H1:H1048576 M80:M81 O80:O81 Q80:Q81">
     <cfRule type="containsText" dxfId="6" priority="3" operator="containsText" text="例行維護中">
       <formula>NOT(ISERROR(SEARCH("例行維護中",D1)))</formula>
     </cfRule>

</xml_diff>